<commit_message>
Build atualizado das planilhas
</commit_message>
<xml_diff>
--- a/dist/data/saldo-devedor.xlsx
+++ b/dist/data/saldo-devedor.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rssla\Desktop\SPE JARDIM LUZ\01. Relatorio Obra Ramon Gerenciamento\meu-dashboard\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rssla\Dropbox\SPE JARDIM LUZ\Gerenciamento de Obra - Ramon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9250AAB5-23ED-4FDC-BF18-98CE69E2722F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15F2469D-9B37-49FC-A5B7-36760CB103B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -462,8 +462,8 @@
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="000"/>
-    <numFmt numFmtId="166" formatCode="###,##0.00"/>
-    <numFmt numFmtId="167" formatCode="##,##0.00"/>
+    <numFmt numFmtId="165" formatCode="###,##0.00"/>
+    <numFmt numFmtId="166" formatCode="##,##0.00"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -498,7 +498,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -534,30 +534,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="hair">
-        <color rgb="FF010000"/>
-      </top>
-      <bottom style="hair">
-        <color rgb="FF010000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="hair">
-        <color rgb="FF010000"/>
-      </right>
-      <top style="hair">
-        <color rgb="FF010000"/>
-      </top>
-      <bottom style="hair">
-        <color rgb="FF010000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -568,47 +544,32 @@
     <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="6" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -953,2603 +914,1816 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M79"/>
+  <dimension ref="A1:G79"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="5.5546875" customWidth="1"/>
-    <col min="3" max="3" width="2.6640625" customWidth="1"/>
-    <col min="4" max="4" width="5.44140625" customWidth="1"/>
-    <col min="5" max="5" width="4.109375" customWidth="1"/>
-    <col min="6" max="6" width="2.6640625" customWidth="1"/>
-    <col min="7" max="7" width="5.44140625" customWidth="1"/>
-    <col min="8" max="8" width="11" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="2.6640625" customWidth="1"/>
-    <col min="12" max="12" width="8.21875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="34.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:7" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="5"/>
-      <c r="H1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6"/>
-      <c r="L1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+    <row r="2" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="12">
+      <c r="B2" s="6">
         <v>101</v>
       </c>
-      <c r="E2" s="13"/>
-      <c r="F2" s="10" t="s">
+      <c r="C2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="G2" s="11"/>
-      <c r="H2" s="1">
+      <c r="D2" s="1">
         <v>330315.8</v>
       </c>
-      <c r="I2" s="7">
+      <c r="E2" s="8">
         <v>373155.9</v>
       </c>
-      <c r="J2" s="8"/>
-      <c r="K2" s="9"/>
-      <c r="L2" s="3">
+      <c r="F2" s="3">
         <v>31616.89</v>
       </c>
-      <c r="M2" s="1">
+      <c r="G2" s="1">
         <v>341629.12</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
+    <row r="3" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="14"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="12">
+      <c r="B3" s="6">
         <v>102</v>
       </c>
-      <c r="E3" s="13"/>
-      <c r="F3" s="10" t="s">
+      <c r="C3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="11"/>
-      <c r="H3" s="1">
+      <c r="D3" s="1">
         <v>298059.74</v>
       </c>
-      <c r="I3" s="7">
+      <c r="E3" s="8">
         <v>339905.81</v>
       </c>
-      <c r="J3" s="8"/>
-      <c r="K3" s="9"/>
-      <c r="L3" s="3">
+      <c r="F3" s="3">
         <v>27861.33</v>
       </c>
-      <c r="M3" s="1">
+      <c r="G3" s="1">
         <v>312116.21999999997</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
+    <row r="4" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="14"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="12">
+      <c r="B4" s="6">
         <v>108</v>
       </c>
-      <c r="E4" s="13"/>
-      <c r="F4" s="10" t="s">
+      <c r="C4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="11"/>
-      <c r="H4" s="1">
+      <c r="D4" s="1">
         <v>337748.12</v>
       </c>
-      <c r="I4" s="7">
+      <c r="E4" s="8">
         <v>338610.88</v>
       </c>
-      <c r="J4" s="8"/>
-      <c r="K4" s="9"/>
-      <c r="L4" s="3">
+      <c r="F4" s="3">
         <v>5596.84</v>
       </c>
-      <c r="M4" s="1">
+      <c r="G4" s="1">
         <v>333014.03999999998</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
+    <row r="5" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="12">
+      <c r="B5" s="6">
         <v>201</v>
       </c>
-      <c r="E5" s="13"/>
-      <c r="F5" s="10" t="s">
+      <c r="C5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="11"/>
-      <c r="H5" s="1">
+      <c r="D5" s="1">
         <v>351450</v>
       </c>
-      <c r="I5" s="7">
+      <c r="E5" s="8">
         <v>351814.2</v>
       </c>
-      <c r="J5" s="8"/>
-      <c r="K5" s="9"/>
-      <c r="L5" s="3">
+      <c r="F5" s="3">
         <v>1046.45</v>
       </c>
-      <c r="M5" s="1">
+      <c r="G5" s="1">
         <v>350767.75</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="14"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="12">
+      <c r="B6" s="6">
         <v>202</v>
       </c>
-      <c r="E6" s="13"/>
-      <c r="F6" s="10" t="s">
+      <c r="C6" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="11"/>
-      <c r="H6" s="1">
+      <c r="D6" s="1">
         <v>297440.3</v>
       </c>
-      <c r="I6" s="7">
+      <c r="E6" s="8">
         <v>341962.4</v>
       </c>
-      <c r="J6" s="8"/>
-      <c r="K6" s="9"/>
-      <c r="L6" s="3">
+      <c r="F6" s="3">
         <v>31695.39</v>
       </c>
-      <c r="M6" s="1">
+      <c r="G6" s="1">
         <v>310287.48</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
+    <row r="7" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="14"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="12">
+      <c r="B7" s="6">
         <v>203</v>
       </c>
-      <c r="E7" s="13"/>
-      <c r="F7" s="10" t="s">
+      <c r="C7" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="11"/>
-      <c r="H7" s="1">
+      <c r="D7" s="1">
         <v>331760.92</v>
       </c>
-      <c r="I7" s="7">
+      <c r="E7" s="8">
         <v>375382.81</v>
       </c>
-      <c r="J7" s="8"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="3">
+      <c r="F7" s="3">
         <v>35824.639999999999</v>
       </c>
-      <c r="M7" s="1">
+      <c r="G7" s="1">
         <v>339823.7</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
+    <row r="8" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="14"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="12">
+      <c r="B8" s="6">
         <v>204</v>
       </c>
-      <c r="E8" s="13"/>
-      <c r="F8" s="10" t="s">
+      <c r="C8" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="G8" s="11"/>
-      <c r="H8" s="1">
+      <c r="D8" s="1">
         <v>331038.36</v>
       </c>
-      <c r="I8" s="7">
+      <c r="E8" s="8">
         <v>371699.15</v>
       </c>
-      <c r="J8" s="8"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="3">
+      <c r="F8" s="3">
         <v>55732.33</v>
       </c>
-      <c r="M8" s="1">
+      <c r="G8" s="1">
         <v>316171.96000000002</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
+    <row r="9" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="12">
+      <c r="B9" s="6">
         <v>205</v>
       </c>
-      <c r="E9" s="13"/>
-      <c r="F9" s="10" t="s">
+      <c r="C9" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G9" s="11"/>
-      <c r="H9" s="1">
+      <c r="D9" s="1">
         <v>297708.18</v>
       </c>
-      <c r="I9" s="7">
+      <c r="E9" s="8">
         <v>341212.55</v>
       </c>
-      <c r="J9" s="8"/>
-      <c r="K9" s="9"/>
-      <c r="L9" s="3">
+      <c r="F9" s="3">
         <v>30286.35</v>
       </c>
-      <c r="M9" s="1">
+      <c r="G9" s="1">
         <v>310943.93</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
+    <row r="10" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="14"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="12">
+      <c r="B10" s="6">
         <v>206</v>
       </c>
-      <c r="E10" s="13"/>
-      <c r="F10" s="10" t="s">
+      <c r="C10" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="G10" s="11"/>
-      <c r="H10" s="1">
+      <c r="D10" s="1">
         <v>312549.92</v>
       </c>
-      <c r="I10" s="7">
+      <c r="E10" s="8">
         <v>356329.05</v>
       </c>
-      <c r="J10" s="8"/>
-      <c r="K10" s="9"/>
-      <c r="L10" s="3">
+      <c r="F10" s="3">
         <v>32181.51</v>
       </c>
-      <c r="M10" s="1">
+      <c r="G10" s="1">
         <v>324230.8</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
+    <row r="11" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="12">
+      <c r="B11" s="6">
         <v>207</v>
       </c>
-      <c r="E11" s="13"/>
-      <c r="F11" s="10" t="s">
+      <c r="C11" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G11" s="11"/>
-      <c r="H11" s="1">
+      <c r="D11" s="1">
         <v>301440</v>
       </c>
-      <c r="I11" s="7">
+      <c r="E11" s="8">
         <v>345489.51</v>
       </c>
-      <c r="J11" s="8"/>
-      <c r="K11" s="9"/>
-      <c r="L11" s="3">
+      <c r="F11" s="3">
         <v>32477.9</v>
       </c>
-      <c r="M11" s="1">
+      <c r="G11" s="1">
         <v>314375.09000000003</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
+    <row r="12" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="14"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="12">
+      <c r="B12" s="6">
         <v>208</v>
       </c>
-      <c r="E12" s="13"/>
-      <c r="F12" s="10" t="s">
+      <c r="C12" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G12" s="11"/>
-      <c r="H12" s="1">
+      <c r="D12" s="1">
         <v>298038.75</v>
       </c>
-      <c r="I12" s="7">
+      <c r="E12" s="8">
         <v>341591.24</v>
       </c>
-      <c r="J12" s="8"/>
-      <c r="K12" s="9"/>
-      <c r="L12" s="3">
+      <c r="F12" s="3">
         <v>28598.29</v>
       </c>
-      <c r="M12" s="1">
+      <c r="G12" s="1">
         <v>313841.98</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="10" t="s">
+    <row r="13" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="14"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="12">
+      <c r="B13" s="6">
         <v>302</v>
       </c>
-      <c r="E13" s="13"/>
-      <c r="F13" s="10" t="s">
+      <c r="C13" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="G13" s="11"/>
-      <c r="H13" s="1">
+      <c r="D13" s="1">
         <v>332171.26</v>
       </c>
-      <c r="I13" s="7">
+      <c r="E13" s="8">
         <v>377742.89</v>
       </c>
-      <c r="J13" s="8"/>
-      <c r="K13" s="9"/>
-      <c r="L13" s="3">
+      <c r="F13" s="3">
         <v>71363.520000000004</v>
       </c>
-      <c r="M13" s="1">
+      <c r="G13" s="1">
         <v>306379.43</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
+    <row r="14" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="14"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="12">
+      <c r="B14" s="6">
         <v>303</v>
       </c>
-      <c r="E14" s="13"/>
-      <c r="F14" s="10" t="s">
+      <c r="C14" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="G14" s="11"/>
-      <c r="H14" s="1">
+      <c r="D14" s="1">
         <v>332171.26</v>
       </c>
-      <c r="I14" s="7">
+      <c r="E14" s="8">
         <v>375710.98</v>
       </c>
-      <c r="J14" s="8"/>
-      <c r="K14" s="9"/>
-      <c r="L14" s="3">
+      <c r="F14" s="3">
         <v>49155.02</v>
       </c>
-      <c r="M14" s="1">
+      <c r="G14" s="1">
         <v>326555.84000000003</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="10" t="s">
+    <row r="15" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="14"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="12">
+      <c r="B15" s="6">
         <v>305</v>
       </c>
-      <c r="E15" s="13"/>
-      <c r="F15" s="10" t="s">
+      <c r="C15" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="G15" s="11"/>
-      <c r="H15" s="1">
+      <c r="D15" s="1">
         <v>330268.78999999998</v>
       </c>
-      <c r="I15" s="7">
+      <c r="E15" s="8">
         <v>375007</v>
       </c>
-      <c r="J15" s="8"/>
-      <c r="K15" s="9"/>
-      <c r="L15" s="3">
+      <c r="F15" s="3">
         <v>34897.85</v>
       </c>
-      <c r="M15" s="1">
+      <c r="G15" s="1">
         <v>340281.97</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="10" t="s">
+    <row r="16" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B16" s="14"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="12">
+      <c r="B16" s="6">
         <v>307</v>
       </c>
-      <c r="E16" s="13"/>
-      <c r="F16" s="10" t="s">
+      <c r="C16" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G16" s="11"/>
-      <c r="H16" s="1">
+      <c r="D16" s="1">
         <v>312960</v>
       </c>
-      <c r="I16" s="7">
+      <c r="E16" s="8">
         <v>358693.17</v>
       </c>
-      <c r="J16" s="8"/>
-      <c r="K16" s="9"/>
-      <c r="L16" s="3">
+      <c r="F16" s="3">
         <v>32442.73</v>
       </c>
-      <c r="M16" s="1">
+      <c r="G16" s="1">
         <v>326389.62</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
+    <row r="17" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B17" s="14"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="12">
+      <c r="B17" s="6">
         <v>308</v>
       </c>
-      <c r="E17" s="13"/>
-      <c r="F17" s="10" t="s">
+      <c r="C17" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="G17" s="11"/>
-      <c r="H17" s="1">
+      <c r="D17" s="1">
         <v>302905.59999999998</v>
       </c>
-      <c r="I17" s="7">
+      <c r="E17" s="8">
         <v>346234.49</v>
       </c>
-      <c r="J17" s="8"/>
-      <c r="K17" s="9"/>
-      <c r="L17" s="3">
+      <c r="F17" s="3">
         <v>26511.18</v>
       </c>
-      <c r="M17" s="1">
+      <c r="G17" s="1">
         <v>319723.25</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="10" t="s">
+    <row r="18" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B18" s="14"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="12">
+      <c r="B18" s="6">
         <v>401</v>
       </c>
-      <c r="E18" s="13"/>
-      <c r="F18" s="10" t="s">
+      <c r="C18" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="G18" s="11"/>
-      <c r="H18" s="1">
+      <c r="D18" s="1">
         <v>340000</v>
       </c>
-      <c r="I18" s="7">
+      <c r="E18" s="8">
         <v>340000</v>
       </c>
-      <c r="J18" s="8"/>
-      <c r="K18" s="9"/>
-      <c r="L18" s="3">
+      <c r="F18" s="3">
         <v>0</v>
       </c>
-      <c r="M18" s="1">
+      <c r="G18" s="1">
         <v>340000</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
+    <row r="19" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B19" s="14"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="12">
+      <c r="B19" s="6">
         <v>403</v>
       </c>
-      <c r="E19" s="13"/>
-      <c r="F19" s="10" t="s">
+      <c r="C19" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="G19" s="11"/>
-      <c r="H19" s="1">
+      <c r="D19" s="1">
         <v>325123.86</v>
       </c>
-      <c r="I19" s="7">
+      <c r="E19" s="8">
         <v>372634.49</v>
       </c>
-      <c r="J19" s="8"/>
-      <c r="K19" s="9"/>
-      <c r="L19" s="3">
+      <c r="F19" s="3">
         <v>29017.06</v>
       </c>
-      <c r="M19" s="1">
+      <c r="G19" s="1">
         <v>344120.49</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="10" t="s">
+    <row r="20" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B20" s="14"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="12">
+      <c r="B20" s="6">
         <v>408</v>
       </c>
-      <c r="E20" s="13"/>
-      <c r="F20" s="10" t="s">
+      <c r="C20" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="G20" s="11"/>
-      <c r="H20" s="1">
+      <c r="D20" s="1">
         <v>303262.8</v>
       </c>
-      <c r="I20" s="7">
+      <c r="E20" s="8">
         <v>347578.73</v>
       </c>
-      <c r="J20" s="8"/>
-      <c r="K20" s="9"/>
-      <c r="L20" s="3">
+      <c r="F20" s="3">
         <v>30502.51</v>
       </c>
-      <c r="M20" s="1">
+      <c r="G20" s="1">
         <v>317076.21999999997</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="10" t="s">
+    <row r="21" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B21" s="14"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="12">
+      <c r="B21" s="6">
         <v>501</v>
       </c>
-      <c r="E21" s="13"/>
-      <c r="F21" s="10" t="s">
+      <c r="C21" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="G21" s="11"/>
-      <c r="H21" s="1">
+      <c r="D21" s="1">
         <v>329769.02</v>
       </c>
-      <c r="I21" s="7">
+      <c r="E21" s="8">
         <v>377758.36</v>
       </c>
-      <c r="J21" s="8"/>
-      <c r="K21" s="9"/>
-      <c r="L21" s="3">
+      <c r="F21" s="3">
         <v>54921.13</v>
       </c>
-      <c r="M21" s="1">
+      <c r="G21" s="1">
         <v>322884.59999999998</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="10" t="s">
+    <row r="22" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B22" s="14"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="12">
+      <c r="B22" s="6">
         <v>502</v>
       </c>
-      <c r="E22" s="13"/>
-      <c r="F22" s="10" t="s">
+      <c r="C22" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G22" s="11"/>
-      <c r="H22" s="1">
+      <c r="D22" s="1">
         <v>326181.05</v>
       </c>
-      <c r="I22" s="7">
+      <c r="E22" s="8">
         <v>373257.56</v>
       </c>
-      <c r="J22" s="8"/>
-      <c r="K22" s="9"/>
-      <c r="L22" s="3">
+      <c r="F22" s="3">
         <v>28945.53</v>
       </c>
-      <c r="M22" s="1">
+      <c r="G22" s="1">
         <v>344662.83</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
+    <row r="23" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B23" s="14"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="12">
+      <c r="B23" s="6">
         <v>504</v>
       </c>
-      <c r="E23" s="13"/>
-      <c r="F23" s="10" t="s">
+      <c r="C23" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="G23" s="11"/>
-      <c r="H23" s="1">
+      <c r="D23" s="1">
         <v>303620</v>
       </c>
-      <c r="I23" s="7">
+      <c r="E23" s="8">
         <v>347050.91</v>
       </c>
-      <c r="J23" s="8"/>
-      <c r="K23" s="9"/>
-      <c r="L23" s="3">
+      <c r="F23" s="3">
         <v>29058.84</v>
       </c>
-      <c r="M23" s="1">
+      <c r="G23" s="1">
         <v>318007.84999999998</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="10" t="s">
+    <row r="24" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B24" s="14"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="12">
+      <c r="B24" s="6">
         <v>505</v>
       </c>
-      <c r="E24" s="13"/>
-      <c r="F24" s="10" t="s">
+      <c r="C24" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="G24" s="11"/>
-      <c r="H24" s="1">
+      <c r="D24" s="1">
         <v>310764</v>
       </c>
-      <c r="I24" s="7">
+      <c r="E24" s="8">
         <v>356300.93</v>
       </c>
-      <c r="J24" s="8"/>
-      <c r="K24" s="9"/>
-      <c r="L24" s="3">
+      <c r="F24" s="3">
         <v>33269.96</v>
       </c>
-      <c r="M24" s="1">
+      <c r="G24" s="1">
         <v>323031.03999999998</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="10" t="s">
+    <row r="25" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B25" s="14"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="12">
+      <c r="B25" s="6">
         <v>506</v>
       </c>
-      <c r="E25" s="13"/>
-      <c r="F25" s="10" t="s">
+      <c r="C25" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="G25" s="11"/>
-      <c r="H25" s="1">
+      <c r="D25" s="1">
         <v>323419.90000000002</v>
       </c>
-      <c r="I25" s="7">
+      <c r="E25" s="8">
         <v>369203.25</v>
       </c>
-      <c r="J25" s="8"/>
-      <c r="K25" s="9"/>
-      <c r="L25" s="3">
+      <c r="F25" s="3">
         <v>20034.7</v>
       </c>
-      <c r="M25" s="1">
+      <c r="G25" s="1">
         <v>349312.2</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="10" t="s">
+    <row r="26" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B26" s="14"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="12">
+      <c r="B26" s="6">
         <v>507</v>
       </c>
-      <c r="E26" s="13"/>
-      <c r="F26" s="10" t="s">
+      <c r="C26" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="G26" s="11"/>
-      <c r="H26" s="1">
+      <c r="D26" s="1">
         <v>309763.71999999997</v>
       </c>
-      <c r="I26" s="7">
+      <c r="E26" s="8">
         <v>354219.91</v>
       </c>
-      <c r="J26" s="8"/>
-      <c r="K26" s="9"/>
-      <c r="L26" s="3">
+      <c r="F26" s="3">
         <v>32392.79</v>
       </c>
-      <c r="M26" s="1">
+      <c r="G26" s="1">
         <v>322131.46999999997</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="10" t="s">
+    <row r="27" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B27" s="14"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="12">
+      <c r="B27" s="6">
         <v>508</v>
       </c>
-      <c r="E27" s="13"/>
-      <c r="F27" s="10" t="s">
+      <c r="C27" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="G27" s="11"/>
-      <c r="H27" s="1">
+      <c r="D27" s="1">
         <v>303831.12</v>
       </c>
-      <c r="I27" s="7">
+      <c r="E27" s="8">
         <v>347988.23</v>
       </c>
-      <c r="J27" s="8"/>
-      <c r="K27" s="9"/>
-      <c r="L27" s="3">
+      <c r="F27" s="3">
         <v>25529.78</v>
       </c>
-      <c r="M27" s="1">
+      <c r="G27" s="1">
         <v>322458.38</v>
       </c>
     </row>
-    <row r="28" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="10" t="s">
+    <row r="28" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="B28" s="14"/>
-      <c r="C28" s="11"/>
-      <c r="D28" s="12">
+      <c r="B28" s="6">
         <v>601</v>
       </c>
-      <c r="E28" s="13"/>
-      <c r="F28" s="10" t="s">
+      <c r="C28" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="G28" s="11"/>
-      <c r="H28" s="1">
+      <c r="D28" s="1">
         <v>341646.88</v>
       </c>
-      <c r="I28" s="7">
+      <c r="E28" s="8">
         <v>350028.41</v>
       </c>
-      <c r="J28" s="8"/>
-      <c r="K28" s="9"/>
-      <c r="L28" s="3">
+      <c r="F28" s="3">
         <v>216915.16</v>
       </c>
-      <c r="M28" s="1">
+      <c r="G28" s="1">
         <v>133196.35999999999</v>
       </c>
     </row>
-    <row r="29" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="10" t="s">
+    <row r="29" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B29" s="14"/>
-      <c r="C29" s="11"/>
-      <c r="D29" s="12">
+      <c r="B29" s="6">
         <v>602</v>
       </c>
-      <c r="E29" s="13"/>
-      <c r="F29" s="10" t="s">
+      <c r="C29" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G29" s="11"/>
-      <c r="H29" s="1">
+      <c r="D29" s="1">
         <v>312906.25</v>
       </c>
-      <c r="I29" s="7">
+      <c r="E29" s="8">
         <v>358631.32</v>
       </c>
-      <c r="J29" s="8"/>
-      <c r="K29" s="9"/>
-      <c r="L29" s="3">
+      <c r="F29" s="3">
         <v>31166.49</v>
       </c>
-      <c r="M29" s="1">
+      <c r="G29" s="1">
         <v>328128.44</v>
       </c>
     </row>
-    <row r="30" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="10" t="s">
+    <row r="30" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B30" s="14"/>
-      <c r="C30" s="11"/>
-      <c r="D30" s="12">
+      <c r="B30" s="6">
         <v>603</v>
       </c>
-      <c r="E30" s="13"/>
-      <c r="F30" s="10" t="s">
+      <c r="C30" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G30" s="11"/>
-      <c r="H30" s="1">
+      <c r="D30" s="1">
         <v>312907.2</v>
       </c>
-      <c r="I30" s="7">
+      <c r="E30" s="8">
         <v>359004.84</v>
       </c>
-      <c r="J30" s="8"/>
-      <c r="K30" s="9"/>
-      <c r="L30" s="3">
+      <c r="F30" s="3">
         <v>34811.18</v>
       </c>
-      <c r="M30" s="1">
+      <c r="G30" s="1">
         <v>324272.63</v>
       </c>
     </row>
-    <row r="31" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="10" t="s">
+    <row r="31" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="B31" s="14"/>
-      <c r="C31" s="11"/>
-      <c r="D31" s="12">
+      <c r="B31" s="6">
         <v>604</v>
       </c>
-      <c r="E31" s="13"/>
-      <c r="F31" s="10" t="s">
+      <c r="C31" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="G31" s="11"/>
-      <c r="H31" s="1">
+      <c r="D31" s="1">
         <v>302977.2</v>
       </c>
-      <c r="I31" s="7">
+      <c r="E31" s="8">
         <v>345544.21</v>
       </c>
-      <c r="J31" s="8"/>
-      <c r="K31" s="9"/>
-      <c r="L31" s="3">
+      <c r="F31" s="3">
         <v>31416.63</v>
       </c>
-      <c r="M31" s="1">
+      <c r="G31" s="1">
         <v>314478.57</v>
       </c>
     </row>
-    <row r="32" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="10" t="s">
+    <row r="32" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="B32" s="14"/>
-      <c r="C32" s="11"/>
-      <c r="D32" s="12">
+      <c r="B32" s="6">
         <v>606</v>
       </c>
-      <c r="E32" s="13"/>
-      <c r="F32" s="10" t="s">
+      <c r="C32" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G32" s="11"/>
-      <c r="H32" s="1">
+      <c r="D32" s="1">
         <v>357976.63</v>
       </c>
-      <c r="I32" s="7">
+      <c r="E32" s="8">
         <v>367254.47</v>
       </c>
-      <c r="J32" s="8"/>
-      <c r="K32" s="9"/>
-      <c r="L32" s="3">
+      <c r="F32" s="3">
         <v>28710.07</v>
       </c>
-      <c r="M32" s="1">
+      <c r="G32" s="1">
         <v>338809.05</v>
       </c>
     </row>
-    <row r="33" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="10" t="s">
+    <row r="33" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B33" s="14"/>
-      <c r="C33" s="11"/>
-      <c r="D33" s="12">
+      <c r="B33" s="6">
         <v>607</v>
       </c>
-      <c r="E33" s="13"/>
-      <c r="F33" s="10" t="s">
+      <c r="C33" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="G33" s="11"/>
-      <c r="H33" s="1">
+      <c r="D33" s="1">
         <v>311121.2</v>
       </c>
-      <c r="I33" s="7">
+      <c r="E33" s="8">
         <v>356710.69</v>
       </c>
-      <c r="J33" s="8"/>
-      <c r="K33" s="9"/>
-      <c r="L33" s="3">
+      <c r="F33" s="3">
         <v>37435.9</v>
       </c>
-      <c r="M33" s="1">
+      <c r="G33" s="1">
         <v>319354.67</v>
       </c>
     </row>
-    <row r="34" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="10" t="s">
+    <row r="34" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="B34" s="14"/>
-      <c r="C34" s="11"/>
-      <c r="D34" s="12">
+      <c r="B34" s="6">
         <v>701</v>
       </c>
-      <c r="E34" s="13"/>
-      <c r="F34" s="10" t="s">
+      <c r="C34" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="G34" s="11"/>
-      <c r="H34" s="1">
+      <c r="D34" s="1">
         <v>311615.64</v>
       </c>
-      <c r="I34" s="7">
+      <c r="E34" s="8">
         <v>357928.58</v>
       </c>
-      <c r="J34" s="8"/>
-      <c r="K34" s="9"/>
-      <c r="L34" s="3">
+      <c r="F34" s="3">
         <v>40732.230000000003</v>
       </c>
-      <c r="M34" s="1">
+      <c r="G34" s="1">
         <v>317196.44</v>
       </c>
     </row>
-    <row r="35" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="10" t="s">
+    <row r="35" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="B35" s="14"/>
-      <c r="C35" s="11"/>
-      <c r="D35" s="12">
+      <c r="B35" s="6">
         <v>703</v>
       </c>
-      <c r="E35" s="13"/>
-      <c r="F35" s="10" t="s">
+      <c r="C35" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G35" s="11"/>
-      <c r="H35" s="1">
+      <c r="D35" s="1">
         <v>311615.64</v>
       </c>
-      <c r="I35" s="7">
+      <c r="E35" s="8">
         <v>357765.74</v>
       </c>
-      <c r="J35" s="8"/>
-      <c r="K35" s="9"/>
-      <c r="L35" s="3">
+      <c r="F35" s="3">
         <v>32412.06</v>
       </c>
-      <c r="M35" s="1">
+      <c r="G35" s="1">
         <v>325385.53999999998</v>
       </c>
     </row>
-    <row r="36" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="10" t="s">
+    <row r="36" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B36" s="14"/>
-      <c r="C36" s="11"/>
-      <c r="D36" s="12">
+      <c r="B36" s="6">
         <v>705</v>
       </c>
-      <c r="E36" s="13"/>
-      <c r="F36" s="10" t="s">
+      <c r="C36" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="G36" s="11"/>
-      <c r="H36" s="1">
+      <c r="D36" s="1">
         <v>312314.15999999997</v>
       </c>
-      <c r="I36" s="7">
+      <c r="E36" s="8">
         <v>358078.49</v>
       </c>
-      <c r="J36" s="8"/>
-      <c r="K36" s="9"/>
-      <c r="L36" s="3">
+      <c r="F36" s="3">
         <v>33483.01</v>
       </c>
-      <c r="M36" s="1">
+      <c r="G36" s="1">
         <v>324642.5</v>
       </c>
     </row>
-    <row r="37" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="10" t="s">
+    <row r="37" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="B37" s="14"/>
-      <c r="C37" s="11"/>
-      <c r="D37" s="12">
+      <c r="B37" s="6">
         <v>708</v>
       </c>
-      <c r="E37" s="13"/>
-      <c r="F37" s="10" t="s">
+      <c r="C37" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="G37" s="11"/>
-      <c r="H37" s="1">
+      <c r="D37" s="1">
         <v>303570.15000000002</v>
       </c>
-      <c r="I37" s="7">
+      <c r="E37" s="8">
         <v>346886.06</v>
       </c>
-      <c r="J37" s="8"/>
-      <c r="K37" s="9"/>
-      <c r="L37" s="3">
+      <c r="F37" s="3">
         <v>33984.74</v>
       </c>
-      <c r="M37" s="1">
+      <c r="G37" s="1">
         <v>312984.03999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="10" t="s">
+    <row r="38" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="B38" s="14"/>
-      <c r="C38" s="11"/>
-      <c r="D38" s="12">
+      <c r="B38" s="6">
         <v>801</v>
       </c>
-      <c r="E38" s="13"/>
-      <c r="F38" s="10" t="s">
+      <c r="C38" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G38" s="11"/>
-      <c r="H38" s="1">
+      <c r="D38" s="1">
         <v>311970.98</v>
       </c>
-      <c r="I38" s="7">
+      <c r="E38" s="8">
         <v>358340.51</v>
       </c>
-      <c r="J38" s="8"/>
-      <c r="K38" s="9"/>
-      <c r="L38" s="3">
+      <c r="F38" s="3">
         <v>40711.51</v>
       </c>
-      <c r="M38" s="1">
+      <c r="G38" s="1">
         <v>317629.07</v>
       </c>
     </row>
-    <row r="39" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="10" t="s">
+    <row r="39" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B39" s="14"/>
-      <c r="C39" s="11"/>
-      <c r="D39" s="12">
+      <c r="B39" s="6">
         <v>803</v>
       </c>
-      <c r="E39" s="13"/>
-      <c r="F39" s="10" t="s">
+      <c r="C39" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G39" s="11"/>
-      <c r="H39" s="1">
+      <c r="D39" s="1">
         <v>312621.65000000002</v>
       </c>
-      <c r="I39" s="7">
+      <c r="E39" s="8">
         <v>357340.34</v>
       </c>
-      <c r="J39" s="8"/>
-      <c r="K39" s="9"/>
-      <c r="L39" s="3">
+      <c r="F39" s="3">
         <v>23898.07</v>
       </c>
-      <c r="M39" s="1">
+      <c r="G39" s="1">
         <v>333744.5</v>
       </c>
     </row>
-    <row r="40" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="10" t="s">
+    <row r="40" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="B40" s="14"/>
-      <c r="C40" s="11"/>
-      <c r="D40" s="12">
+      <c r="B40" s="6">
         <v>805</v>
       </c>
-      <c r="E40" s="13"/>
-      <c r="F40" s="10" t="s">
+      <c r="C40" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G40" s="11"/>
-      <c r="H40" s="1">
+      <c r="D40" s="1">
         <v>338365.6</v>
       </c>
-      <c r="I40" s="7">
+      <c r="E40" s="8">
         <v>347375.22</v>
       </c>
-      <c r="J40" s="8"/>
-      <c r="K40" s="9"/>
-      <c r="L40" s="3">
+      <c r="F40" s="3">
         <v>215794</v>
       </c>
-      <c r="M40" s="1">
+      <c r="G40" s="1">
         <v>131581.28</v>
       </c>
     </row>
-    <row r="41" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="10" t="s">
+    <row r="41" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="B41" s="14"/>
-      <c r="C41" s="11"/>
-      <c r="D41" s="12">
+      <c r="B41" s="6">
         <v>807</v>
       </c>
-      <c r="E41" s="13"/>
-      <c r="F41" s="10" t="s">
+      <c r="C41" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="G41" s="11"/>
-      <c r="H41" s="1">
+      <c r="D41" s="1">
         <v>362848.43</v>
       </c>
-      <c r="I41" s="7">
+      <c r="E41" s="8">
         <v>374386.07</v>
       </c>
-      <c r="J41" s="8"/>
-      <c r="K41" s="9"/>
-      <c r="L41" s="3">
+      <c r="F41" s="3">
         <v>88780.160000000003</v>
       </c>
-      <c r="M41" s="1">
+      <c r="G41" s="1">
         <v>285345.49</v>
       </c>
     </row>
-    <row r="42" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="10" t="s">
+    <row r="42" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="B42" s="14"/>
-      <c r="C42" s="11"/>
-      <c r="D42" s="12">
+      <c r="B42" s="6">
         <v>808</v>
       </c>
-      <c r="E42" s="13"/>
-      <c r="F42" s="10" t="s">
+      <c r="C42" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="G42" s="11"/>
-      <c r="H42" s="1">
+      <c r="D42" s="1">
         <v>304691.59999999998</v>
       </c>
-      <c r="I42" s="7">
+      <c r="E42" s="8">
         <v>349406.28</v>
       </c>
-      <c r="J42" s="8"/>
-      <c r="K42" s="9"/>
-      <c r="L42" s="3">
+      <c r="F42" s="3">
         <v>32440.6</v>
       </c>
-      <c r="M42" s="1">
+      <c r="G42" s="1">
         <v>316980.56</v>
       </c>
     </row>
-    <row r="43" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="10" t="s">
+    <row r="43" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B43" s="14"/>
-      <c r="C43" s="11"/>
-      <c r="D43" s="12">
+      <c r="B43" s="6">
         <v>902</v>
       </c>
-      <c r="E43" s="13"/>
-      <c r="F43" s="10" t="s">
+      <c r="C43" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="G43" s="11"/>
-      <c r="H43" s="1">
+      <c r="D43" s="1">
         <v>290000</v>
       </c>
-      <c r="I43" s="7">
+      <c r="E43" s="8">
         <v>290000</v>
       </c>
-      <c r="J43" s="8"/>
-      <c r="K43" s="9"/>
-      <c r="L43" s="3">
+      <c r="F43" s="3">
         <v>0</v>
       </c>
-      <c r="M43" s="1">
+      <c r="G43" s="1">
         <v>290000</v>
       </c>
     </row>
-    <row r="44" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="10" t="s">
+    <row r="44" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="B44" s="14"/>
-      <c r="C44" s="11"/>
-      <c r="D44" s="12">
+      <c r="B44" s="6">
         <v>903</v>
       </c>
-      <c r="E44" s="13"/>
-      <c r="F44" s="10" t="s">
+      <c r="C44" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="G44" s="11"/>
-      <c r="H44" s="1">
+      <c r="D44" s="1">
         <v>338158.2</v>
       </c>
-      <c r="I44" s="7">
+      <c r="E44" s="8">
         <v>384190.44</v>
       </c>
-      <c r="J44" s="8"/>
-      <c r="K44" s="9"/>
-      <c r="L44" s="3">
+      <c r="F44" s="3">
         <v>40525.83</v>
       </c>
-      <c r="M44" s="1">
+      <c r="G44" s="1">
         <v>343649.94</v>
       </c>
     </row>
-    <row r="45" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="10" t="s">
+    <row r="45" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="B45" s="14"/>
-      <c r="C45" s="11"/>
-      <c r="D45" s="12">
+      <c r="B45" s="6">
         <v>907</v>
       </c>
-      <c r="E45" s="13"/>
-      <c r="F45" s="10" t="s">
+      <c r="C45" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="G45" s="11"/>
-      <c r="H45" s="1">
+      <c r="D45" s="1">
         <v>311121.2</v>
       </c>
-      <c r="I45" s="7">
+      <c r="E45" s="8">
         <v>357690.95</v>
       </c>
-      <c r="J45" s="8"/>
-      <c r="K45" s="9"/>
-      <c r="L45" s="3">
+      <c r="F45" s="3">
         <v>33646.15</v>
       </c>
-      <c r="M45" s="1">
+      <c r="G45" s="1">
         <v>324044.75</v>
       </c>
     </row>
-    <row r="46" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="10" t="s">
+    <row r="46" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="B46" s="14"/>
-      <c r="C46" s="11"/>
-      <c r="D46" s="12">
+      <c r="B46" s="6">
         <v>908</v>
       </c>
-      <c r="E46" s="13"/>
-      <c r="F46" s="10" t="s">
+      <c r="C46" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="G46" s="11"/>
-      <c r="H46" s="1">
+      <c r="D46" s="1">
         <v>307727.76</v>
       </c>
-      <c r="I46" s="7">
+      <c r="E46" s="8">
         <v>352819.73</v>
       </c>
-      <c r="J46" s="8"/>
-      <c r="K46" s="9"/>
-      <c r="L46" s="3">
+      <c r="F46" s="3">
         <v>39367.79</v>
       </c>
-      <c r="M46" s="1">
+      <c r="G46" s="1">
         <v>313451.99</v>
       </c>
     </row>
-    <row r="47" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="10" t="s">
+    <row r="47" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="B47" s="14"/>
-      <c r="C47" s="11"/>
-      <c r="D47" s="12">
+      <c r="B47" s="6">
         <v>1001</v>
       </c>
-      <c r="E47" s="13"/>
-      <c r="F47" s="10" t="s">
+      <c r="C47" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="G47" s="11"/>
-      <c r="H47" s="1">
+      <c r="D47" s="1">
         <v>321153</v>
       </c>
-      <c r="I47" s="7">
+      <c r="E47" s="8">
         <v>366475.21</v>
       </c>
-      <c r="J47" s="8"/>
-      <c r="K47" s="9"/>
-      <c r="L47" s="3">
+      <c r="F47" s="3">
         <v>45917.71</v>
       </c>
-      <c r="M47" s="1">
+      <c r="G47" s="1">
         <v>320732.09999999998</v>
       </c>
     </row>
-    <row r="48" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="10" t="s">
+    <row r="48" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="B48" s="14"/>
-      <c r="C48" s="11"/>
-      <c r="D48" s="12">
+      <c r="B48" s="6">
         <v>1003</v>
       </c>
-      <c r="E48" s="13"/>
-      <c r="F48" s="10" t="s">
+      <c r="C48" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="G48" s="11"/>
-      <c r="H48" s="1">
+      <c r="D48" s="1">
         <v>360355.93</v>
       </c>
-      <c r="I48" s="7">
+      <c r="E48" s="8">
         <v>398892.9</v>
       </c>
-      <c r="J48" s="8"/>
-      <c r="K48" s="9"/>
-      <c r="L48" s="3">
+      <c r="F48" s="3">
         <v>19808.490000000002</v>
       </c>
-      <c r="M48" s="1">
+      <c r="G48" s="1">
         <v>379709.97</v>
       </c>
     </row>
-    <row r="49" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="10" t="s">
+    <row r="49" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="B49" s="14"/>
-      <c r="C49" s="11"/>
-      <c r="D49" s="12">
+      <c r="B49" s="6">
         <v>1004</v>
       </c>
-      <c r="E49" s="13"/>
-      <c r="F49" s="10" t="s">
+      <c r="C49" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="G49" s="11"/>
-      <c r="H49" s="1">
+      <c r="D49" s="1">
         <v>310493</v>
       </c>
-      <c r="I49" s="7">
+      <c r="E49" s="8">
         <v>355865.4</v>
       </c>
-      <c r="J49" s="8"/>
-      <c r="K49" s="9"/>
-      <c r="L49" s="3">
+      <c r="F49" s="3">
         <v>40365.089999999997</v>
       </c>
-      <c r="M49" s="1">
+      <c r="G49" s="1">
         <v>315531.75</v>
       </c>
     </row>
-    <row r="50" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="10" t="s">
+    <row r="50" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="B50" s="14"/>
-      <c r="C50" s="11"/>
-      <c r="D50" s="12">
+      <c r="B50" s="6">
         <v>1005</v>
       </c>
-      <c r="E50" s="13"/>
-      <c r="F50" s="10" t="s">
+      <c r="C50" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="G50" s="11"/>
-      <c r="H50" s="1">
+      <c r="D50" s="1">
         <v>347641.85</v>
       </c>
-      <c r="I50" s="7">
+      <c r="E50" s="8">
         <v>379260.75</v>
       </c>
-      <c r="J50" s="8"/>
-      <c r="K50" s="9"/>
-      <c r="L50" s="3">
+      <c r="F50" s="3">
         <v>33494.93</v>
       </c>
-      <c r="M50" s="1">
+      <c r="G50" s="1">
         <v>346351.37</v>
       </c>
     </row>
-    <row r="51" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="10" t="s">
+    <row r="51" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="B51" s="14"/>
-      <c r="C51" s="11"/>
-      <c r="D51" s="12">
+      <c r="B51" s="6">
         <v>1007</v>
       </c>
-      <c r="E51" s="13"/>
-      <c r="F51" s="10" t="s">
+      <c r="C51" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="G51" s="11"/>
-      <c r="H51" s="1">
+      <c r="D51" s="1">
         <v>360000</v>
       </c>
-      <c r="I51" s="7">
+      <c r="E51" s="8">
         <v>360546.5</v>
       </c>
-      <c r="J51" s="8"/>
-      <c r="K51" s="9"/>
-      <c r="L51" s="3">
+      <c r="F51" s="3">
         <v>1562.74</v>
       </c>
-      <c r="M51" s="1">
+      <c r="G51" s="1">
         <v>358983.76</v>
       </c>
     </row>
-    <row r="52" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="10" t="s">
+    <row r="52" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="B52" s="14"/>
-      <c r="C52" s="11"/>
-      <c r="D52" s="12">
+      <c r="B52" s="6">
         <v>1102</v>
       </c>
-      <c r="E52" s="13"/>
-      <c r="F52" s="10" t="s">
+      <c r="C52" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="G52" s="11"/>
-      <c r="H52" s="1">
+      <c r="D52" s="1">
         <v>338400</v>
       </c>
-      <c r="I52" s="7">
+      <c r="E52" s="8">
         <v>339767.42</v>
       </c>
-      <c r="J52" s="8"/>
-      <c r="K52" s="9"/>
-      <c r="L52" s="3">
+      <c r="F52" s="3">
         <v>7168.19</v>
       </c>
-      <c r="M52" s="1">
+      <c r="G52" s="1">
         <v>332603.53000000003</v>
       </c>
     </row>
-    <row r="53" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="10" t="s">
+    <row r="53" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="B53" s="14"/>
-      <c r="C53" s="11"/>
-      <c r="D53" s="12">
+      <c r="B53" s="6">
         <v>1107</v>
       </c>
-      <c r="E53" s="13"/>
-      <c r="F53" s="10" t="s">
+      <c r="C53" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="G53" s="11"/>
-      <c r="H53" s="1">
+      <c r="D53" s="1">
         <v>357200</v>
       </c>
-      <c r="I53" s="7">
+      <c r="E53" s="8">
         <v>357200</v>
       </c>
-      <c r="J53" s="8"/>
-      <c r="K53" s="9"/>
-      <c r="L53" s="3">
+      <c r="F53" s="3">
         <v>77200</v>
       </c>
-      <c r="M53" s="1">
+      <c r="G53" s="1">
         <v>280000</v>
       </c>
     </row>
-    <row r="54" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="10" t="s">
+    <row r="54" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="B54" s="14"/>
-      <c r="C54" s="11"/>
-      <c r="D54" s="12">
+      <c r="B54" s="6">
         <v>1108</v>
       </c>
-      <c r="E54" s="13"/>
-      <c r="F54" s="10" t="s">
+      <c r="C54" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="G54" s="11"/>
-      <c r="H54" s="1">
+      <c r="D54" s="1">
         <v>370000</v>
       </c>
-      <c r="I54" s="7">
+      <c r="E54" s="8">
         <v>370000</v>
       </c>
-      <c r="J54" s="8"/>
-      <c r="K54" s="9"/>
-      <c r="L54" s="3">
+      <c r="F54" s="3">
         <v>1000</v>
       </c>
-      <c r="M54" s="1">
+      <c r="G54" s="1">
         <v>369000</v>
       </c>
     </row>
-    <row r="55" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="10" t="s">
+    <row r="55" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="B55" s="14"/>
-      <c r="C55" s="11"/>
-      <c r="D55" s="12">
+      <c r="B55" s="6">
         <v>1201</v>
       </c>
-      <c r="E55" s="13"/>
-      <c r="F55" s="10" t="s">
+      <c r="C55" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="G55" s="11"/>
-      <c r="H55" s="1">
+      <c r="D55" s="1">
         <v>358027</v>
       </c>
-      <c r="I55" s="7">
+      <c r="E55" s="8">
         <v>389918.88</v>
       </c>
-      <c r="J55" s="8"/>
-      <c r="K55" s="9"/>
-      <c r="L55" s="3">
+      <c r="F55" s="3">
         <v>33078.5</v>
       </c>
-      <c r="M55" s="1">
+      <c r="G55" s="1">
         <v>357556.57</v>
       </c>
     </row>
-    <row r="56" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="10" t="s">
+    <row r="56" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="B56" s="14"/>
-      <c r="C56" s="11"/>
-      <c r="D56" s="12">
+      <c r="B56" s="6">
         <v>1202</v>
       </c>
-      <c r="E56" s="13"/>
-      <c r="F56" s="10" t="s">
+      <c r="C56" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="G56" s="11"/>
-      <c r="H56" s="1">
+      <c r="D56" s="1">
         <v>338400</v>
       </c>
-      <c r="I56" s="7">
+      <c r="E56" s="8">
         <v>339302.49</v>
       </c>
-      <c r="J56" s="8"/>
-      <c r="K56" s="9"/>
-      <c r="L56" s="3">
+      <c r="F56" s="3">
         <v>2295.7199999999998</v>
       </c>
-      <c r="M56" s="1">
+      <c r="G56" s="1">
         <v>337006.77</v>
       </c>
     </row>
-    <row r="57" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="10" t="s">
+    <row r="57" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="B57" s="14"/>
-      <c r="C57" s="11"/>
-      <c r="D57" s="12">
+      <c r="B57" s="6">
         <v>1204</v>
       </c>
-      <c r="E57" s="13"/>
-      <c r="F57" s="10" t="s">
+      <c r="C57" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="G57" s="11"/>
-      <c r="H57" s="1">
+      <c r="D57" s="1">
         <v>312445.5</v>
       </c>
-      <c r="I57" s="7">
+      <c r="E57" s="8">
         <v>359213.45</v>
       </c>
-      <c r="J57" s="8"/>
-      <c r="K57" s="9"/>
-      <c r="L57" s="3">
+      <c r="F57" s="3">
         <v>32325.34</v>
       </c>
-      <c r="M57" s="1">
+      <c r="G57" s="1">
         <v>326908.26</v>
       </c>
     </row>
-    <row r="58" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="10" t="s">
+    <row r="58" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="B58" s="14"/>
-      <c r="C58" s="11"/>
-      <c r="D58" s="12">
+      <c r="B58" s="6">
         <v>1206</v>
       </c>
-      <c r="E58" s="13"/>
-      <c r="F58" s="10" t="s">
+      <c r="C58" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="G58" s="11"/>
-      <c r="H58" s="1">
+      <c r="D58" s="1">
         <v>312445.5</v>
       </c>
-      <c r="I58" s="7">
+      <c r="E58" s="8">
         <v>359213.45</v>
       </c>
-      <c r="J58" s="8"/>
-      <c r="K58" s="9"/>
-      <c r="L58" s="3">
+      <c r="F58" s="3">
         <v>31599.16</v>
       </c>
-      <c r="M58" s="1">
+      <c r="G58" s="1">
         <v>327785.17</v>
       </c>
     </row>
-    <row r="59" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="10" t="s">
+    <row r="59" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B59" s="14"/>
-      <c r="C59" s="11"/>
-      <c r="D59" s="12">
+      <c r="B59" s="6">
         <v>1207</v>
       </c>
-      <c r="E59" s="13"/>
-      <c r="F59" s="10" t="s">
+      <c r="C59" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="G59" s="11"/>
-      <c r="H59" s="1">
+      <c r="D59" s="1">
         <v>336490</v>
       </c>
-      <c r="I59" s="7">
+      <c r="E59" s="8">
         <v>381253.85</v>
       </c>
-      <c r="J59" s="8"/>
-      <c r="K59" s="9"/>
-      <c r="L59" s="3">
+      <c r="F59" s="3">
         <v>67390.820000000007</v>
       </c>
-      <c r="M59" s="1">
+      <c r="G59" s="1">
         <v>314843.84999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="10" t="s">
+    <row r="60" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="B60" s="14"/>
-      <c r="C60" s="11"/>
-      <c r="D60" s="12">
+      <c r="B60" s="6">
         <v>1208</v>
       </c>
-      <c r="E60" s="13"/>
-      <c r="F60" s="10" t="s">
+      <c r="C60" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="G60" s="11"/>
-      <c r="H60" s="1">
+      <c r="D60" s="1">
         <v>370000</v>
       </c>
-      <c r="I60" s="7">
+      <c r="E60" s="8">
         <v>370596.82</v>
       </c>
-      <c r="J60" s="8"/>
-      <c r="K60" s="9"/>
-      <c r="L60" s="3">
+      <c r="F60" s="3">
         <v>1975.24</v>
       </c>
-      <c r="M60" s="1">
+      <c r="G60" s="1">
         <v>368621.58</v>
       </c>
     </row>
-    <row r="61" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="10" t="s">
+    <row r="61" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B61" s="14"/>
-      <c r="C61" s="11"/>
-      <c r="D61" s="12">
+      <c r="B61" s="6">
         <v>1301</v>
       </c>
-      <c r="E61" s="13"/>
-      <c r="F61" s="10" t="s">
+      <c r="C61" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="G61" s="11"/>
-      <c r="H61" s="1">
+      <c r="D61" s="1">
         <v>264000</v>
       </c>
-      <c r="I61" s="7">
+      <c r="E61" s="8">
         <v>264000</v>
       </c>
-      <c r="J61" s="8"/>
-      <c r="K61" s="9"/>
-      <c r="L61" s="3">
+      <c r="F61" s="3">
         <v>0</v>
       </c>
-      <c r="M61" s="1">
+      <c r="G61" s="1">
         <v>264000</v>
       </c>
     </row>
-    <row r="62" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="10" t="s">
+    <row r="62" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="B62" s="14"/>
-      <c r="C62" s="11"/>
-      <c r="D62" s="12">
+      <c r="B62" s="6">
         <v>1302</v>
       </c>
-      <c r="E62" s="13"/>
-      <c r="F62" s="10" t="s">
+      <c r="C62" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="G62" s="11"/>
-      <c r="H62" s="1">
+      <c r="D62" s="1">
         <v>307598.46999999997</v>
       </c>
-      <c r="I62" s="7">
+      <c r="E62" s="8">
         <v>316906.26</v>
       </c>
-      <c r="J62" s="8"/>
-      <c r="K62" s="9"/>
-      <c r="L62" s="3">
+      <c r="F62" s="3">
         <v>306835</v>
       </c>
-      <c r="M62" s="1">
+      <c r="G62" s="1">
         <v>10234.15</v>
       </c>
     </row>
-    <row r="63" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="10" t="s">
+    <row r="63" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="B63" s="14"/>
-      <c r="C63" s="11"/>
-      <c r="D63" s="12">
+      <c r="B63" s="6">
         <v>1304</v>
       </c>
-      <c r="E63" s="13"/>
-      <c r="F63" s="10" t="s">
+      <c r="C63" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="G63" s="11"/>
-      <c r="H63" s="1">
+      <c r="D63" s="1">
         <v>312425.51</v>
       </c>
-      <c r="I63" s="7">
+      <c r="E63" s="8">
         <v>358400.07</v>
       </c>
-      <c r="J63" s="8"/>
-      <c r="K63" s="9"/>
-      <c r="L63" s="3">
+      <c r="F63" s="3">
         <v>32281.52</v>
       </c>
-      <c r="M63" s="1">
+      <c r="G63" s="1">
         <v>326996.44</v>
       </c>
     </row>
-    <row r="64" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="10" t="s">
+    <row r="64" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="B64" s="14"/>
-      <c r="C64" s="11"/>
-      <c r="D64" s="12">
+      <c r="B64" s="6">
         <v>1306</v>
       </c>
-      <c r="E64" s="13"/>
-      <c r="F64" s="10" t="s">
+      <c r="C64" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="G64" s="11"/>
-      <c r="H64" s="1">
+      <c r="D64" s="1">
         <v>353485.55</v>
       </c>
-      <c r="I64" s="7">
+      <c r="E64" s="8">
         <v>358682.47</v>
       </c>
-      <c r="J64" s="8"/>
-      <c r="K64" s="9"/>
-      <c r="L64" s="3">
+      <c r="F64" s="3">
         <v>232292.64</v>
       </c>
-      <c r="M64" s="1">
+      <c r="G64" s="1">
         <v>126528.42</v>
       </c>
     </row>
-    <row r="65" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="10" t="s">
+    <row r="65" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B65" s="14"/>
-      <c r="C65" s="11"/>
-      <c r="D65" s="12">
+      <c r="B65" s="6">
         <v>1307</v>
       </c>
-      <c r="E65" s="13"/>
-      <c r="F65" s="10" t="s">
+      <c r="C65" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="G65" s="11"/>
-      <c r="H65" s="1">
+      <c r="D65" s="1">
         <v>357200</v>
       </c>
-      <c r="I65" s="7">
+      <c r="E65" s="8">
         <v>357493.92</v>
       </c>
-      <c r="J65" s="8"/>
-      <c r="K65" s="9"/>
-      <c r="L65" s="3">
+      <c r="F65" s="3">
         <v>28260.639999999999</v>
       </c>
-      <c r="M65" s="1">
+      <c r="G65" s="1">
         <v>329233.28000000003</v>
       </c>
     </row>
-    <row r="66" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="10" t="s">
+    <row r="66" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="B66" s="14"/>
-      <c r="C66" s="11"/>
-      <c r="D66" s="12">
+      <c r="B66" s="6">
         <v>1308</v>
       </c>
-      <c r="E66" s="13"/>
-      <c r="F66" s="10" t="s">
+      <c r="C66" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="G66" s="11"/>
-      <c r="H66" s="1">
+      <c r="D66" s="1">
         <v>312806.5</v>
       </c>
-      <c r="I66" s="7">
+      <c r="E66" s="8">
         <v>358642.94</v>
       </c>
-      <c r="J66" s="8"/>
-      <c r="K66" s="9"/>
-      <c r="L66" s="3">
+      <c r="F66" s="3">
         <v>33331.410000000003</v>
       </c>
-      <c r="M66" s="1">
+      <c r="G66" s="1">
         <v>325346.28000000003</v>
       </c>
     </row>
-    <row r="67" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="10" t="s">
+    <row r="67" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="B67" s="14"/>
-      <c r="C67" s="11"/>
-      <c r="D67" s="12">
+      <c r="B67" s="6">
         <v>1401</v>
       </c>
-      <c r="E67" s="13"/>
-      <c r="F67" s="10" t="s">
+      <c r="C67" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="G67" s="11"/>
-      <c r="H67" s="1">
+      <c r="D67" s="1">
         <v>264000</v>
       </c>
-      <c r="I67" s="7">
+      <c r="E67" s="8">
         <v>264000</v>
       </c>
-      <c r="J67" s="8"/>
-      <c r="K67" s="9"/>
-      <c r="L67" s="3">
+      <c r="F67" s="3">
         <v>0</v>
       </c>
-      <c r="M67" s="1">
+      <c r="G67" s="1">
         <v>264000</v>
       </c>
     </row>
-    <row r="68" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="10" t="s">
+    <row r="68" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="B68" s="14"/>
-      <c r="C68" s="11"/>
-      <c r="D68" s="12">
+      <c r="B68" s="6">
         <v>1402</v>
       </c>
-      <c r="E68" s="13"/>
-      <c r="F68" s="10" t="s">
+      <c r="C68" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="G68" s="11"/>
-      <c r="H68" s="1">
+      <c r="D68" s="1">
         <v>370782.5</v>
       </c>
-      <c r="I68" s="7">
+      <c r="E68" s="8">
         <v>408799.46</v>
       </c>
-      <c r="J68" s="8"/>
-      <c r="K68" s="9"/>
-      <c r="L68" s="3">
+      <c r="F68" s="3">
         <v>43509.9</v>
       </c>
-      <c r="M68" s="1">
+      <c r="G68" s="1">
         <v>367535.8</v>
       </c>
     </row>
-    <row r="69" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="10" t="s">
+    <row r="69" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="B69" s="14"/>
-      <c r="C69" s="11"/>
-      <c r="D69" s="12">
+      <c r="B69" s="6">
         <v>1406</v>
       </c>
-      <c r="E69" s="13"/>
-      <c r="F69" s="10" t="s">
+      <c r="C69" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="G69" s="11"/>
-      <c r="H69" s="1">
+      <c r="D69" s="1">
         <v>322710</v>
       </c>
-      <c r="I69" s="7">
+      <c r="E69" s="8">
         <v>369867.89</v>
       </c>
-      <c r="J69" s="8"/>
-      <c r="K69" s="9"/>
-      <c r="L69" s="3">
+      <c r="F69" s="3">
         <v>29730.05</v>
       </c>
-      <c r="M69" s="1">
+      <c r="G69" s="1">
         <v>340938.92</v>
       </c>
     </row>
-    <row r="70" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="10" t="s">
+    <row r="70" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="B70" s="14"/>
-      <c r="C70" s="11"/>
-      <c r="D70" s="12">
+      <c r="B70" s="6">
         <v>1407</v>
       </c>
-      <c r="E70" s="13"/>
-      <c r="F70" s="10" t="s">
+      <c r="C70" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="G70" s="11"/>
-      <c r="H70" s="1">
+      <c r="D70" s="1">
         <v>336688.35</v>
       </c>
-      <c r="I70" s="7">
+      <c r="E70" s="8">
         <v>383500.59</v>
       </c>
-      <c r="J70" s="8"/>
-      <c r="K70" s="9"/>
-      <c r="L70" s="3">
+      <c r="F70" s="3">
         <v>39818.080000000002</v>
       </c>
-      <c r="M70" s="1">
+      <c r="G70" s="1">
         <v>343682.56</v>
       </c>
     </row>
-    <row r="71" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="10" t="s">
+    <row r="71" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="B71" s="14"/>
-      <c r="C71" s="11"/>
-      <c r="D71" s="12">
+      <c r="B71" s="6">
         <v>1408</v>
       </c>
-      <c r="E71" s="13"/>
-      <c r="F71" s="10" t="s">
+      <c r="C71" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="G71" s="11"/>
-      <c r="H71" s="1">
+      <c r="D71" s="1">
         <v>370000</v>
       </c>
-      <c r="I71" s="7">
+      <c r="E71" s="8">
         <v>370000</v>
       </c>
-      <c r="J71" s="8"/>
-      <c r="K71" s="9"/>
-      <c r="L71" s="3">
+      <c r="F71" s="3">
         <v>0</v>
       </c>
-      <c r="M71" s="1">
+      <c r="G71" s="1">
         <v>370000</v>
       </c>
     </row>
-    <row r="72" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="10" t="s">
+    <row r="72" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A72" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="B72" s="14"/>
-      <c r="C72" s="11"/>
-      <c r="D72" s="12">
+      <c r="B72" s="6">
         <v>1501</v>
       </c>
-      <c r="E72" s="13"/>
-      <c r="F72" s="10" t="s">
+      <c r="C72" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="G72" s="11"/>
-      <c r="H72" s="1">
+      <c r="D72" s="1">
         <v>330407</v>
       </c>
-      <c r="I72" s="7">
+      <c r="E72" s="8">
         <v>372559.1</v>
       </c>
-      <c r="J72" s="8"/>
-      <c r="K72" s="9"/>
-      <c r="L72" s="3">
+      <c r="F72" s="3">
         <v>83987.45</v>
       </c>
-      <c r="M72" s="1">
+      <c r="G72" s="1">
         <v>289911.77</v>
       </c>
     </row>
-    <row r="73" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="10" t="s">
+    <row r="73" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A73" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="B73" s="14"/>
-      <c r="C73" s="11"/>
-      <c r="D73" s="12">
+      <c r="B73" s="6">
         <v>1502</v>
       </c>
-      <c r="E73" s="13"/>
-      <c r="F73" s="10" t="s">
+      <c r="C73" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="G73" s="11"/>
-      <c r="H73" s="1">
+      <c r="D73" s="1">
         <v>370000</v>
       </c>
-      <c r="I73" s="7">
+      <c r="E73" s="8">
         <v>370710.73</v>
       </c>
-      <c r="J73" s="8"/>
-      <c r="K73" s="9"/>
-      <c r="L73" s="3">
+      <c r="F73" s="3">
         <v>6383.49</v>
       </c>
-      <c r="M73" s="1">
+      <c r="G73" s="1">
         <v>364327.23</v>
       </c>
     </row>
-    <row r="74" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="10" t="s">
+    <row r="74" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="B74" s="14"/>
-      <c r="C74" s="11"/>
-      <c r="D74" s="12">
+      <c r="B74" s="6">
         <v>1503</v>
       </c>
-      <c r="E74" s="13"/>
-      <c r="F74" s="10" t="s">
+      <c r="C74" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="G74" s="11"/>
-      <c r="H74" s="1">
+      <c r="D74" s="1">
         <v>318801.02</v>
       </c>
-      <c r="I74" s="7">
+      <c r="E74" s="8">
         <v>365515.77</v>
       </c>
-      <c r="J74" s="8"/>
-      <c r="K74" s="9"/>
-      <c r="L74" s="3">
+      <c r="F74" s="3">
         <v>35501.839999999997</v>
       </c>
-      <c r="M74" s="1">
+      <c r="G74" s="1">
         <v>330438.78999999998</v>
       </c>
     </row>
-    <row r="75" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="10" t="s">
+    <row r="75" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="B75" s="14"/>
-      <c r="C75" s="11"/>
-      <c r="D75" s="12">
+      <c r="B75" s="6">
         <v>1505</v>
       </c>
-      <c r="E75" s="13"/>
-      <c r="F75" s="10" t="s">
+      <c r="C75" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="G75" s="11"/>
-      <c r="H75" s="1">
+      <c r="D75" s="1">
         <v>319060.34000000003</v>
       </c>
-      <c r="I75" s="7">
+      <c r="E75" s="8">
         <v>366060.12</v>
       </c>
-      <c r="J75" s="8"/>
-      <c r="K75" s="9"/>
-      <c r="L75" s="3">
+      <c r="F75" s="3">
         <v>33218.99</v>
       </c>
-      <c r="M75" s="1">
+      <c r="G75" s="1">
         <v>332886.07</v>
       </c>
     </row>
-    <row r="76" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="10" t="s">
+    <row r="76" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="B76" s="14"/>
-      <c r="C76" s="11"/>
-      <c r="D76" s="12">
+      <c r="B76" s="6">
         <v>1506</v>
       </c>
-      <c r="E76" s="13"/>
-      <c r="F76" s="10" t="s">
+      <c r="C76" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="G76" s="11"/>
-      <c r="H76" s="1">
+      <c r="D76" s="1">
         <v>332138.32</v>
       </c>
-      <c r="I76" s="7">
+      <c r="E76" s="8">
         <v>343223.33</v>
       </c>
-      <c r="J76" s="8"/>
-      <c r="K76" s="9"/>
-      <c r="L76" s="3">
+      <c r="F76" s="3">
         <v>262674.77</v>
       </c>
-      <c r="M76" s="1">
+      <c r="G76" s="1">
         <v>74591.64</v>
       </c>
     </row>
-    <row r="77" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="10" t="s">
+    <row r="77" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="B77" s="14"/>
-      <c r="C77" s="11"/>
-      <c r="D77" s="12">
+      <c r="B77" s="6">
         <v>1507</v>
       </c>
-      <c r="E77" s="13"/>
-      <c r="F77" s="10" t="s">
+      <c r="C77" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G77" s="11"/>
-      <c r="H77" s="1">
+      <c r="D77" s="1">
         <v>327356.09999999998</v>
       </c>
-      <c r="I77" s="7">
+      <c r="E77" s="8">
         <v>335485.38</v>
       </c>
-      <c r="J77" s="8"/>
-      <c r="K77" s="9"/>
-      <c r="L77" s="3">
+      <c r="F77" s="3">
         <v>224847.35</v>
       </c>
-      <c r="M77" s="1">
+      <c r="G77" s="1">
         <v>110629.74</v>
       </c>
     </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A78" s="10" t="s">
+    <row r="78" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="B78" s="14"/>
-      <c r="C78" s="11"/>
-      <c r="D78" s="12">
+      <c r="B78" s="6">
         <v>1508</v>
       </c>
-      <c r="E78" s="13"/>
-      <c r="F78" s="10" t="s">
+      <c r="C78" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="G78" s="11"/>
-      <c r="H78" s="1">
+      <c r="D78" s="1">
         <v>347800</v>
       </c>
-      <c r="I78" s="7">
+      <c r="E78" s="8">
         <v>348166.36</v>
       </c>
-      <c r="J78" s="8"/>
-      <c r="K78" s="9"/>
-      <c r="L78" s="3">
+      <c r="F78" s="3">
         <v>0</v>
       </c>
-      <c r="M78" s="1">
+      <c r="G78" s="1">
         <v>348166.36</v>
       </c>
     </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="I79" s="4"/>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E79" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="312">
-    <mergeCell ref="A77:C77"/>
-    <mergeCell ref="D77:E77"/>
-    <mergeCell ref="F77:G77"/>
-    <mergeCell ref="I77:K77"/>
-    <mergeCell ref="A78:C78"/>
-    <mergeCell ref="D78:E78"/>
-    <mergeCell ref="F78:G78"/>
-    <mergeCell ref="I78:K78"/>
-    <mergeCell ref="A76:C76"/>
-    <mergeCell ref="D76:E76"/>
-    <mergeCell ref="F76:G76"/>
-    <mergeCell ref="I76:K76"/>
-    <mergeCell ref="A73:C73"/>
-    <mergeCell ref="D73:E73"/>
-    <mergeCell ref="F73:G73"/>
-    <mergeCell ref="I73:K73"/>
-    <mergeCell ref="A74:C74"/>
-    <mergeCell ref="D74:E74"/>
-    <mergeCell ref="F74:G74"/>
-    <mergeCell ref="I74:K74"/>
-    <mergeCell ref="A75:C75"/>
-    <mergeCell ref="D75:E75"/>
-    <mergeCell ref="F75:G75"/>
-    <mergeCell ref="I75:K75"/>
-    <mergeCell ref="A70:C70"/>
-    <mergeCell ref="D70:E70"/>
-    <mergeCell ref="F70:G70"/>
-    <mergeCell ref="I70:K70"/>
-    <mergeCell ref="A71:C71"/>
-    <mergeCell ref="D71:E71"/>
-    <mergeCell ref="F71:G71"/>
-    <mergeCell ref="I71:K71"/>
-    <mergeCell ref="A72:C72"/>
-    <mergeCell ref="D72:E72"/>
-    <mergeCell ref="F72:G72"/>
-    <mergeCell ref="I72:K72"/>
-    <mergeCell ref="A67:C67"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="F67:G67"/>
-    <mergeCell ref="I67:K67"/>
-    <mergeCell ref="A68:C68"/>
-    <mergeCell ref="D68:E68"/>
-    <mergeCell ref="F68:G68"/>
-    <mergeCell ref="I68:K68"/>
-    <mergeCell ref="A69:C69"/>
-    <mergeCell ref="D69:E69"/>
-    <mergeCell ref="F69:G69"/>
-    <mergeCell ref="I69:K69"/>
-    <mergeCell ref="A64:C64"/>
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="F64:G64"/>
-    <mergeCell ref="I64:K64"/>
-    <mergeCell ref="A65:C65"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="F65:G65"/>
-    <mergeCell ref="I65:K65"/>
-    <mergeCell ref="A66:C66"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="F66:G66"/>
-    <mergeCell ref="I66:K66"/>
-    <mergeCell ref="A61:C61"/>
-    <mergeCell ref="D61:E61"/>
-    <mergeCell ref="F61:G61"/>
-    <mergeCell ref="I61:K61"/>
-    <mergeCell ref="A62:C62"/>
-    <mergeCell ref="D62:E62"/>
-    <mergeCell ref="F62:G62"/>
-    <mergeCell ref="I62:K62"/>
-    <mergeCell ref="A63:C63"/>
-    <mergeCell ref="D63:E63"/>
-    <mergeCell ref="F63:G63"/>
-    <mergeCell ref="I63:K63"/>
-    <mergeCell ref="A58:C58"/>
-    <mergeCell ref="D58:E58"/>
-    <mergeCell ref="F58:G58"/>
-    <mergeCell ref="I58:K58"/>
-    <mergeCell ref="A59:C59"/>
-    <mergeCell ref="D59:E59"/>
-    <mergeCell ref="F59:G59"/>
-    <mergeCell ref="I59:K59"/>
-    <mergeCell ref="A60:C60"/>
-    <mergeCell ref="D60:E60"/>
-    <mergeCell ref="F60:G60"/>
-    <mergeCell ref="I60:K60"/>
-    <mergeCell ref="A55:C55"/>
-    <mergeCell ref="D55:E55"/>
-    <mergeCell ref="F55:G55"/>
-    <mergeCell ref="I55:K55"/>
-    <mergeCell ref="A56:C56"/>
-    <mergeCell ref="D56:E56"/>
-    <mergeCell ref="F56:G56"/>
-    <mergeCell ref="I56:K56"/>
-    <mergeCell ref="A57:C57"/>
-    <mergeCell ref="D57:E57"/>
-    <mergeCell ref="F57:G57"/>
-    <mergeCell ref="I57:K57"/>
-    <mergeCell ref="A52:C52"/>
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="F52:G52"/>
-    <mergeCell ref="I52:K52"/>
-    <mergeCell ref="A53:C53"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="F53:G53"/>
-    <mergeCell ref="I53:K53"/>
-    <mergeCell ref="A54:C54"/>
-    <mergeCell ref="D54:E54"/>
-    <mergeCell ref="F54:G54"/>
-    <mergeCell ref="I54:K54"/>
-    <mergeCell ref="A49:C49"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="F49:G49"/>
-    <mergeCell ref="I49:K49"/>
-    <mergeCell ref="A50:C50"/>
-    <mergeCell ref="D50:E50"/>
-    <mergeCell ref="F50:G50"/>
-    <mergeCell ref="I50:K50"/>
-    <mergeCell ref="A51:C51"/>
-    <mergeCell ref="D51:E51"/>
-    <mergeCell ref="F51:G51"/>
-    <mergeCell ref="I51:K51"/>
-    <mergeCell ref="A46:C46"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="F46:G46"/>
-    <mergeCell ref="I46:K46"/>
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="F47:G47"/>
-    <mergeCell ref="I47:K47"/>
-    <mergeCell ref="A48:C48"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="F48:G48"/>
-    <mergeCell ref="I48:K48"/>
-    <mergeCell ref="A43:C43"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="F43:G43"/>
-    <mergeCell ref="I43:K43"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="F44:G44"/>
-    <mergeCell ref="I44:K44"/>
-    <mergeCell ref="A45:C45"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="F45:G45"/>
-    <mergeCell ref="I45:K45"/>
-    <mergeCell ref="A40:C40"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="F40:G40"/>
-    <mergeCell ref="I40:K40"/>
-    <mergeCell ref="A41:C41"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="F41:G41"/>
-    <mergeCell ref="I41:K41"/>
-    <mergeCell ref="A42:C42"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="F42:G42"/>
-    <mergeCell ref="I42:K42"/>
-    <mergeCell ref="A37:C37"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="F37:G37"/>
-    <mergeCell ref="I37:K37"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="F38:G38"/>
-    <mergeCell ref="I38:K38"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="F39:G39"/>
-    <mergeCell ref="I39:K39"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="I34:K34"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="F35:G35"/>
-    <mergeCell ref="I35:K35"/>
-    <mergeCell ref="A36:C36"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="I36:K36"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="I31:K31"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="I33:K33"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="I28:K28"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="I29:K29"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="I30:K30"/>
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="I25:K25"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="I26:K26"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="I27:K27"/>
-    <mergeCell ref="A22:C22"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="I22:K22"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="I23:K23"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="I24:K24"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="I19:K19"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="I20:K20"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="I21:K21"/>
-    <mergeCell ref="A16:C16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="I16:K16"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="I17:K17"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="I18:K18"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="I13:K13"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="I14:K14"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="I15:K15"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="I10:K10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="I11:K11"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="I12:K12"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="I7:K7"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="I9:K9"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="I4:K4"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="I5:K5"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="I6:K6"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="I3:K3"/>
-  </mergeCells>
   <pageMargins left="0.52999994886203072" right="0.52999994886203072" top="0.52999994886203072" bottom="0.68999998212799307" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="landscape"/>
 </worksheet>

</xml_diff>